<commit_message>
Publicar reconstruccion MIP y simulador piloto
</commit_message>
<xml_diff>
--- a/MIP/Mexico/MIP_Mexico_2003.xlsx
+++ b/MIP/Mexico/MIP_Mexico_2003.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="g_produccion" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W_valor_agregado" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="f_demanda_final" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CI_importado" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ajuste_intermedio" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="multiplicadores" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balances_sectoriales" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="validacion_resumen" sheetId="13" state="visible" r:id="rId13"/>
@@ -34,7 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'g_produccion'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'W_valor_agregado'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'f_demanda_final'!$A$1:$B$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CI_importado'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'ajuste_intermedio'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'multiplicadores'!$A$1:$H$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'balances_sectoriales'!$A$1:$M$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'validacion_resumen'!$A$1:$C$12</definedName>
@@ -640,12 +640,12 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>descripcion_CI_importado</t>
+          <t>descripcion_ajuste_intermedio</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Consumo intermedio importado fuera de Z; cierre VA: g = colsum(Z nacional) + CI importado + W.</t>
+          <t>Ajuste intermedio fuera de Z. En MIP directas puede ser CI importado; en COU reconstruidos con puente de precios puede incluir importaciones, margenes, impuestos y diferencias de valoracion comprador-basico.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       <c r="A1" s="2" t="n"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>ci_importado</t>
+          <t>ajuste_intermedio_no_basico</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>consumo_intermedio_importado</t>
+          <t>ajuste_intermedio_no_basico</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>consumo_intermedio_importado</t>
+          <t>ajuste_intermedio_no_basico</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">

</xml_diff>